<commit_message>
Add comprehensive NPI trace feature regression
</commit_message>
<xml_diff>
--- a/tool_all_features_trace_template.xlsx
+++ b/tool_all_features_trace_template.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG4"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -460,28 +460,30 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="17" customWidth="1" min="23" max="23"/>
-    <col width="21" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
-    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="17" customWidth="1" min="25" max="25"/>
+    <col width="21" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
     <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
     <col width="14" customWidth="1" min="30" max="30"/>
-    <col width="14" customWidth="1" min="31" max="31"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
     <col width="14" customWidth="1" min="32" max="32"/>
     <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -542,110 +544,120 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>drv_wide_bit</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>drv_const_direct</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>drv_const_parent</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>drv_const_source</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>drv_noise</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>drv_reg_endpoint</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>drv_ternary_stop</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>drv_float</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>load_bus[7]</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>load_bus[15]</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>load_plain</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>load_module_port</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>load_sibling_bus</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>load_leaf_bus</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>load_reg_endpoint</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>load_unconnected</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>aux_in</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>aux_float</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>aux_out</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>aux_unused_out</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>leaf_in</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>leaf_out</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>in</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>used</t>
         </is>
@@ -689,6 +701,8 @@
       <c r="AE2" s="2" t="n"/>
       <c r="AF2" s="2" t="n"/>
       <c r="AG2" s="2" t="n"/>
+      <c r="AH2" s="2" t="n"/>
+      <c r="AI2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -728,6 +742,8 @@
       <c r="AE3" s="2" t="n"/>
       <c r="AF3" s="2" t="n"/>
       <c r="AG3" s="2" t="n"/>
+      <c r="AH3" s="2" t="n"/>
+      <c r="AI3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -767,6 +783,8 @@
       <c r="AE4" s="2" t="n"/>
       <c r="AF4" s="2" t="n"/>
       <c r="AG4" s="2" t="n"/>
+      <c r="AH4" s="2" t="n"/>
+      <c r="AI4" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>